<commit_message>
Update 500 Excel template: add AutoFilter (pulldown search on 区分/図面名 etc.)
</commit_message>
<xml_diff>
--- a/tokuten500_excel_v0_9beta.xlsx
+++ b/tokuten500_excel_v0_9beta.xlsx
@@ -15,7 +15,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⑤IFC書き出し設定記録" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⑥AI出力検証ログ" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'①法規調査チェック'!$A$4:$H$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'②図面整合チェック'!$A$4:$I$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'③申請図書リスト'!$A$4:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'④関連手続きチェック'!$A$4:$G$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'⑤IFC書き出し設定記録'!$A$4:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'⑥AI出力検証ログ'!$A$4:$G$24</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -2728,6 +2735,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:H76"/>
   <mergeCells count="3">
     <mergeCell ref="A78:H78"/>
     <mergeCell ref="A2:H2"/>
@@ -4669,6 +4677,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:I67"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -5507,6 +5516,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:G36"/>
   <mergeCells count="3">
     <mergeCell ref="A38:G38"/>
     <mergeCell ref="A2:G2"/>
@@ -6178,6 +6188,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:G25"/>
   <mergeCells count="3">
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A2:G2"/>
@@ -6397,6 +6408,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:F13"/>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -6703,6 +6715,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:G24"/>
   <mergeCells count="3">
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A2:G2"/>

</xml_diff>